<commit_message>
🎯 Strike: Label column in upload files
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brand-protection/2026-09-28/strike/00-pilot-5.xlsx
+++ b/brand-protection/2026-09-28/strike/00-pilot-5.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,11 @@
           <t>Tags</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +444,11 @@
           <t>strike-01-mono-other</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -451,6 +461,11 @@
           <t>strike-02-mono-mixed</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -463,6 +478,11 @@
           <t>strike-03-mb-page-other</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -475,6 +495,11 @@
           <t>strike-04-bait</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -485,6 +510,11 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>strike-05-redirect-other</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🎯 Strike: upload files in Corsearch template format (url, label, tags, geo, name)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brand-protection/2026-09-28/strike/00-pilot-5.xlsx
+++ b/brand-protection/2026-09-28/strike/00-pilot-5.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="sample" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,23 +413,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>url</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Tags</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Label</t>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>website_category</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>phone_number</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>email_address</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>wechat</t>
         </is>
       </c>
     </row>
@@ -441,12 +491,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>strike-01-mono-other</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Trademark Infringement</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>100milesofbeskidwyspowy.com</t>
         </is>
       </c>
     </row>
@@ -458,12 +518,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>strike-02-mono-mixed</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Trademark Infringement</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bartlettcabinet.com</t>
         </is>
       </c>
     </row>
@@ -475,12 +545,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>strike-03-mb-page-other</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Trademark Infringement</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>bookmakerslife.ru</t>
         </is>
       </c>
     </row>
@@ -492,12 +572,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>strike-04-bait</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Trademark Infringement</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>24mostbet.click</t>
         </is>
       </c>
     </row>
@@ -509,12 +594,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>strike-05-redirect-other</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Trademark Infringement</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>mostbet-cz.co</t>
         </is>
       </c>
     </row>

</xml_diff>